<commit_message>
Ficha: contrato que termina até jan/2027 em destaque verde
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KVpPvh6XktNZmCmX6XKXyn
</commit_message>
<xml_diff>
--- a/Squad and Budget.xlsx
+++ b/Squad and Budget.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/henriquesimoessilva/Meu Drive/6. arquivos pessoais Henrique/Santa Cruz/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AEB6260-E111-4B49-AE96-096117B927D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D3DC255-8849-DC40-B6BC-D17842359C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17260" xr2:uid="{4E7F6755-7A6F-491B-BBC9-63535A73B458}"/>
+    <workbookView xWindow="33520" yWindow="320" windowWidth="30240" windowHeight="17260" xr2:uid="{4E7F6755-7A6F-491B-BBC9-63535A73B458}"/>
   </bookViews>
   <sheets>
     <sheet name="Squad" sheetId="1" r:id="rId1"/>
@@ -400,7 +400,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -434,6 +434,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF002060"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -490,7 +496,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -531,6 +537,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -823,7 +834,7 @@
       </c>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="20" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -851,7 +862,7 @@
       </c>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="20" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -882,7 +893,7 @@
       </c>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="20" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -922,7 +933,7 @@
       </c>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="20" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -963,7 +974,7 @@
       </c>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="20" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -1004,7 +1015,7 @@
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="20" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -1086,7 +1097,7 @@
       </c>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="20" t="s">
         <v>25</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -1127,7 +1138,7 @@
       </c>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="20" t="s">
         <v>27</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -1170,7 +1181,7 @@
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="20" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -1211,7 +1222,7 @@
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="20" t="s">
         <v>32</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -1433,85 +1444,85 @@
       </c>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="E20" s="3">
+      <c r="E20" s="21">
         <v>58700.232266666666</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="21">
         <v>704402.78720000002</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="G20" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="H20" s="10">
+      <c r="H20" s="22">
         <f t="shared" si="0"/>
         <v>47843.449496342735</v>
       </c>
-      <c r="I20" s="10">
+      <c r="I20" s="22">
         <f t="shared" si="1"/>
         <v>621964.84345245559</v>
       </c>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="E21" s="3">
+      <c r="E21" s="21">
         <v>57700.232266666666</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="21">
         <v>692402.78720000002</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="G21" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="H21" s="10">
+      <c r="H21" s="22">
         <f t="shared" si="0"/>
         <v>47028.402474399161</v>
       </c>
-      <c r="I21" s="10">
+      <c r="I21" s="22">
         <f t="shared" si="1"/>
         <v>611369.23216718913</v>
       </c>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="E22" s="3">
+      <c r="E22" s="21">
         <v>50734.522053333327</v>
       </c>
-      <c r="F22" s="3">
+      <c r="F22" s="21">
         <v>608814.26463999995</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="G22" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="H22" s="10">
+      <c r="H22" s="22">
         <f t="shared" si="0"/>
         <v>41351.021109299887</v>
       </c>
-      <c r="I22" s="10">
+      <c r="I22" s="22">
         <f t="shared" si="1"/>
         <v>537563.27442089852</v>
       </c>
@@ -1585,29 +1596,29 @@
       </c>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E24" s="21">
         <v>39799.275813333334</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F24" s="21">
         <v>477591.30976000003</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="G24" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="H24" s="10">
+      <c r="H24" s="22">
         <f t="shared" si="0"/>
         <v>32438.281227168231</v>
       </c>
-      <c r="I24" s="10">
+      <c r="I24" s="22">
         <f t="shared" si="1"/>
         <v>421697.65595318697</v>
       </c>
@@ -1857,29 +1868,29 @@
       </c>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="E30" s="3">
+      <c r="E30" s="21">
         <v>20900.23782026667</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30" s="21">
         <v>250802.85384320005</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="G30" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="H30" s="10">
+      <c r="H30" s="22">
         <f t="shared" si="0"/>
         <v>17034.676593320797</v>
       </c>
-      <c r="I30" s="10">
+      <c r="I30" s="22">
         <f t="shared" si="1"/>
         <v>221450.79571317037</v>
       </c>
@@ -2232,7 +2243,7 @@
         <v>250000</v>
       </c>
       <c r="N63" s="17">
-        <f>L63*M63</f>
+        <f t="shared" ref="N63:N69" si="12">L63*M63</f>
         <v>250000</v>
       </c>
       <c r="O63" s="17">
@@ -2255,15 +2266,15 @@
         <v>200000</v>
       </c>
       <c r="N64" s="17">
-        <f>L64*M64</f>
+        <f t="shared" si="12"/>
         <v>400000</v>
       </c>
       <c r="O64" s="17">
-        <f t="shared" ref="O64:O68" si="12">N64*13</f>
+        <f t="shared" ref="O64:O68" si="13">N64*13</f>
         <v>5200000</v>
       </c>
       <c r="P64" s="17">
-        <f t="shared" ref="P64:P68" si="13">O64/L64</f>
+        <f t="shared" ref="P64:P68" si="14">O64/L64</f>
         <v>2600000</v>
       </c>
     </row>
@@ -2278,15 +2289,15 @@
         <v>150000</v>
       </c>
       <c r="N65" s="17">
-        <f>L65*M65</f>
+        <f t="shared" si="12"/>
         <v>600000</v>
       </c>
       <c r="O65" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>7800000</v>
       </c>
       <c r="P65" s="17">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1950000</v>
       </c>
     </row>
@@ -2301,15 +2312,15 @@
         <v>100000</v>
       </c>
       <c r="N66" s="17">
-        <f>L66*M66</f>
+        <f t="shared" si="12"/>
         <v>500000</v>
       </c>
       <c r="O66" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>6500000</v>
       </c>
       <c r="P66" s="17">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1300000</v>
       </c>
     </row>
@@ -2324,15 +2335,15 @@
         <v>70000</v>
       </c>
       <c r="N67" s="17">
-        <f>L67*M67</f>
+        <f t="shared" si="12"/>
         <v>350000</v>
       </c>
       <c r="O67" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>4550000</v>
       </c>
       <c r="P67" s="17">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>910000</v>
       </c>
     </row>
@@ -2347,15 +2358,15 @@
         <v>50000</v>
       </c>
       <c r="N68" s="17">
-        <f>L68*M68</f>
+        <f t="shared" si="12"/>
         <v>250000</v>
       </c>
       <c r="O68" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3250000</v>
       </c>
       <c r="P68" s="17">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>650000</v>
       </c>
     </row>
@@ -2370,7 +2381,7 @@
         <v>30000</v>
       </c>
       <c r="N69" s="17">
-        <f>L69*M69</f>
+        <f t="shared" si="12"/>
         <v>120000</v>
       </c>
       <c r="O69" s="17">

</xml_diff>